<commit_message>
Trait conflicts: opposite traits cannot be picked together at creation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/player.xlsx
+++ b/tools/sheets/player.xlsx
@@ -1180,6 +1180,11 @@
           <t>모든 신체 부위 최대 체력 +10%</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>frail_body</t>
+        </is>
+      </c>
       <c r="H4" t="n">
         <v>1</v>
       </c>
@@ -1256,6 +1261,11 @@
           <t>달리기 속도 +10%</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>slow_mover</t>
+        </is>
+      </c>
       <c r="H6" t="n">
         <v>1</v>
       </c>
@@ -1294,6 +1304,11 @@
           <t>회피 액션의 허용 타이밍 범위 증가</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>slow_reflexes</t>
+        </is>
+      </c>
       <c r="H7" t="n">
         <v>1</v>
       </c>
@@ -1375,6 +1390,11 @@
           <t>최대 소지 무게 증가</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>weak_lifter</t>
+        </is>
+      </c>
       <c r="H9" t="n">
         <v>1</v>
       </c>
@@ -1413,6 +1433,11 @@
           <t>포만감 감소 속도 −20%</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>big_eater</t>
+        </is>
+      </c>
       <c r="H10" t="n">
         <v>1</v>
       </c>
@@ -1451,6 +1476,11 @@
           <t>수분 감소 속도 −20%</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>excess_sweating</t>
+        </is>
+      </c>
       <c r="H11" t="n">
         <v>1</v>
       </c>
@@ -1489,6 +1519,11 @@
           <t>수면 회복 효율 증가</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>insomnia, light_sleep</t>
+        </is>
+      </c>
       <c r="H12" t="n">
         <v>1</v>
       </c>
@@ -1527,6 +1562,11 @@
           <t>위생 감소 속도 −20%</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>excess_sweating</t>
+        </is>
+      </c>
       <c r="H13" t="n">
         <v>1</v>
       </c>
@@ -1565,6 +1605,11 @@
           <t>멘탈 감소량 −20%</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>fragile_mind</t>
+        </is>
+      </c>
       <c r="H14" t="n">
         <v>1</v>
       </c>
@@ -1603,6 +1648,11 @@
           <t>괴물 조우 시 공포 상태이상 저항 확률 증가</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>coward</t>
+        </is>
+      </c>
       <c r="H15" t="n">
         <v>1</v>
       </c>
@@ -1684,6 +1734,11 @@
           <t>설득 관련 d20 판정 +2</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>social_misfit</t>
+        </is>
+      </c>
       <c r="H17" t="n">
         <v>1</v>
       </c>
@@ -1722,6 +1777,11 @@
           <t>대화 d20 대실패 위험 완화</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>unlucky</t>
+        </is>
+      </c>
       <c r="H18" t="n">
         <v>0</v>
       </c>
@@ -1965,6 +2025,11 @@
           <t>포만감 감소 속도 +25%</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>light_eater</t>
+        </is>
+      </c>
       <c r="H24" t="n">
         <v>1</v>
       </c>
@@ -2003,6 +2068,11 @@
           <t>수분·위생 감소 속도 증가</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>water_saver, clean_body</t>
+        </is>
+      </c>
       <c r="H25" t="n">
         <v>1</v>
       </c>
@@ -2041,6 +2111,11 @@
           <t>수면 회복 효율 감소</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>sound_sleeper</t>
+        </is>
+      </c>
       <c r="H26" t="n">
         <v>1</v>
       </c>
@@ -2079,6 +2154,11 @@
           <t>수면 중 방해받기 쉬움</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>sound_sleeper</t>
+        </is>
+      </c>
       <c r="H27" t="n">
         <v>0</v>
       </c>
@@ -2122,6 +2202,11 @@
           <t>모든 신체 부위 최대 체력 −10%</t>
         </is>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>robust_body</t>
+        </is>
+      </c>
       <c r="H28" t="n">
         <v>1</v>
       </c>
@@ -2160,6 +2245,11 @@
           <t>최대 소지 무게 감소</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>powerful</t>
+        </is>
+      </c>
       <c r="H29" t="n">
         <v>1</v>
       </c>
@@ -2198,6 +2288,11 @@
           <t>회피 액션 허용 시간 감소</t>
         </is>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>reflexes</t>
+        </is>
+      </c>
       <c r="H30" t="n">
         <v>1</v>
       </c>
@@ -2241,6 +2336,11 @@
           <t>걷기·달리기 속도 −10%</t>
         </is>
       </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>athlete</t>
+        </is>
+      </c>
       <c r="H31" t="n">
         <v>1</v>
       </c>
@@ -2403,6 +2503,11 @@
           <t>괴물 조우 시 멘탈 추가 감소</t>
         </is>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>brave</t>
+        </is>
+      </c>
       <c r="H35" t="n">
         <v>1</v>
       </c>
@@ -2446,6 +2551,11 @@
           <t>멘탈 감소량 +20%</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>iron_mind</t>
+        </is>
+      </c>
       <c r="H36" t="n">
         <v>1</v>
       </c>
@@ -2522,6 +2632,11 @@
           <t>일부 설득·사교 d20 판정 −2</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>persuasive</t>
+        </is>
+      </c>
       <c r="H38" t="n">
         <v>1</v>
       </c>
@@ -2639,6 +2754,11 @@
       <c r="F41" t="inlineStr">
         <is>
           <t>대화 d20 대실패 위험 증가</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>lucky</t>
         </is>
       </c>
       <c r="H41" t="n">
@@ -2730,7 +2850,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>

</xml_diff>